<commit_message>
fix: correct label errors
</commit_message>
<xml_diff>
--- a/data/labels/lesmis_validation.xlsx
+++ b/data/labels/lesmis_validation.xlsx
@@ -8,16 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Startklar\Downloads\archive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18621E4B-DF86-430D-92D9-84D611075729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EF78DFAD-A3AD-496A-A012-55C62CA86B0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C8F467FF-C6E2-4D27-9C34-9166595F527D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{C8F467FF-C6E2-4D27-9C34-9166595F527D}"/>
   </bookViews>
   <sheets>
-    <sheet name="transcript" sheetId="2" r:id="rId1"/>
-    <sheet name="Tabelle1" sheetId="1" r:id="rId2"/>
+    <sheet name="lesmis_validation" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="ExterneDaten_1" localSheetId="0" hidden="1">transcript!$A$1:$D$21</definedName>
+    <definedName name="ExterneDaten_1" localSheetId="0" hidden="1">lesmis_validation!$A$1:$D$21</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="46">
   <si>
     <t>lesmis/lesmis_0001.wav</t>
   </si>
@@ -155,9 +154,6 @@
     <t>lesmis/lesmis_0017.wav</t>
   </si>
   <si>
-    <t>_Fex urbis, lex orbis._</t>
-  </si>
-  <si>
     <t>Fex urbis, lex orbis.</t>
   </si>
   <si>
@@ -165,9 +161,6 @@
   </si>
   <si>
     <t>Les exaspérations de cette foule qui souffre et qui saigne, ses violences à contre-sens sur les principes qui sont sa vie, ses voies de fait contre le droit, sont des coups d'État populaires, et doivent être réprimés.</t>
-  </si>
-  <si>
-    <t>Les exaspérations de cette foule qui souffre et qui saigne, ses violences à contre-sens sur les principes qui sont sa vie, ses voies de fait contre le droit, sont des coups d' tat populaires, et doivent être réprimés.</t>
   </si>
   <si>
     <t>L'homme probe s'y dévoue, et, par amour même pour cette foule, il la combat. Mais comme il la sent excusable tout en lui tenant tête!</t>
@@ -230,9 +223,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -609,30 +601,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9053C34-4577-4EEB-BDB7-A533A52C7ECD}">
   <dimension ref="A1:E21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="44.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="81.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="44.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="81.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" t="s">
         <v>42</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>43</v>
       </c>
-      <c r="C1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>45</v>
       </c>
-      <c r="E1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -645,9 +637,8 @@
       <c r="D2">
         <v>7.63</v>
       </c>
-      <c r="E2" s="1"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -660,9 +651,8 @@
       <c r="D3">
         <v>9.41</v>
       </c>
-      <c r="E3" s="1"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -675,9 +665,8 @@
       <c r="D4">
         <v>6.27</v>
       </c>
-      <c r="E4" s="1"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -690,9 +679,8 @@
       <c r="D5">
         <v>9.24</v>
       </c>
-      <c r="E5" s="1"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -705,9 +693,8 @@
       <c r="D6">
         <v>6.54</v>
       </c>
-      <c r="E6" s="1"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -720,9 +707,8 @@
       <c r="D7">
         <v>14</v>
       </c>
-      <c r="E7" s="1"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -735,9 +721,8 @@
       <c r="D8">
         <v>8.89</v>
       </c>
-      <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -750,9 +735,8 @@
       <c r="D9">
         <v>6.55</v>
       </c>
-      <c r="E9" s="1"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -765,9 +749,8 @@
       <c r="D10">
         <v>9.75</v>
       </c>
-      <c r="E10" s="1"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -780,9 +763,8 @@
       <c r="D11">
         <v>7.67</v>
       </c>
-      <c r="E11" s="1"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -795,9 +777,8 @@
       <c r="D12">
         <v>8.2799999999999994</v>
       </c>
-      <c r="E12" s="1"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -810,9 +791,8 @@
       <c r="D13">
         <v>9.18</v>
       </c>
-      <c r="E13" s="1"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -825,9 +805,8 @@
       <c r="D14">
         <v>8.2899999999999991</v>
       </c>
-      <c r="E14" s="1"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -840,9 +819,8 @@
       <c r="D15">
         <v>5.5</v>
       </c>
-      <c r="E15" s="1"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -855,9 +833,8 @@
       <c r="D16">
         <v>8.18</v>
       </c>
-      <c r="E16" s="1"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>31</v>
       </c>
@@ -870,9 +847,8 @@
       <c r="D17">
         <v>8.7200000000000006</v>
       </c>
-      <c r="E17" s="1"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>33</v>
       </c>
@@ -880,57 +856,53 @@
         <v>34</v>
       </c>
       <c r="C18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D18">
         <v>3.48</v>
       </c>
-      <c r="E18" s="1"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" t="s">
         <v>36</v>
       </c>
-      <c r="B19" t="s">
-        <v>37</v>
-      </c>
       <c r="C19" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D19">
         <v>12.39</v>
       </c>
-      <c r="E19" s="1"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B20" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C20" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D20">
         <v>8.9</v>
       </c>
-      <c r="E20" s="1"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C21" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D21">
         <v>7.52</v>
       </c>
-      <c r="E21" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -938,15 +910,6 @@
   <tableParts count="1">
     <tablePart r:id="rId2"/>
   </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BB44F13-7BDB-4DD2-920E-4078F601306D}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>